<commit_message>
easing the 2040 pet/dsl dropoff
</commit_message>
<xml_diff>
--- a/SysSettings.xlsx
+++ b/SysSettings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_NZL_EECA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E48C51-8FA1-4FE9-9F8D-BB26F26A8EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30803A2C-946C-4D40-BB9F-ABDBFCE2AB60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="F12" s="8" t="str">
         <f t="shared" ref="F12:G12" si="0">"msy"&amp;COUNT(F14:F45)&amp;"_"&amp;MAX(F14:F45)</f>
-        <v>msy6_2030</v>
+        <v>msy13_2050</v>
       </c>
       <c r="G12" s="8" t="str">
         <f t="shared" si="0"/>
@@ -6171,7 +6171,8 @@
         <v>2026</v>
       </c>
       <c r="F16" s="6">
-        <v>2024</v>
+        <f>F15+5</f>
+        <v>2025</v>
       </c>
       <c r="G16" s="6">
         <f>G15+5</f>
@@ -6200,7 +6201,8 @@
         <v>2031</v>
       </c>
       <c r="F17" s="6">
-        <v>2025</v>
+        <f>F16+2</f>
+        <v>2027</v>
       </c>
       <c r="G17" s="6">
         <f>G16+1</f>
@@ -6229,7 +6231,8 @@
         <v>2036</v>
       </c>
       <c r="F18" s="6">
-        <v>2026</v>
+        <f>F17+3</f>
+        <v>2030</v>
       </c>
       <c r="G18" s="6">
         <f t="shared" ref="G18:H26" si="4">G17+1</f>
@@ -6258,7 +6261,8 @@
         <v>2041</v>
       </c>
       <c r="F19" s="6">
-        <v>2030</v>
+        <f>F18+2</f>
+        <v>2032</v>
       </c>
       <c r="G19" s="6">
         <f t="shared" si="4"/>
@@ -6286,6 +6290,10 @@
         <f t="shared" si="3"/>
         <v>2046</v>
       </c>
+      <c r="F20" s="6">
+        <f>F19+3</f>
+        <v>2035</v>
+      </c>
       <c r="G20" s="6">
         <f t="shared" si="4"/>
         <v>2029</v>
@@ -6308,6 +6316,10 @@
       <c r="D21" s="6" t="s">
         <v>46</v>
       </c>
+      <c r="F21" s="6">
+        <f>F20+2</f>
+        <v>2037</v>
+      </c>
       <c r="G21" s="6">
         <f t="shared" si="4"/>
         <v>2030</v>
@@ -6330,6 +6342,10 @@
       <c r="D22" s="6" t="s">
         <v>46</v>
       </c>
+      <c r="F22" s="6">
+        <f>F21+3</f>
+        <v>2040</v>
+      </c>
       <c r="G22" s="6">
         <f t="shared" si="4"/>
         <v>2031</v>
@@ -6352,6 +6368,10 @@
       <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
+      <c r="F23" s="6">
+        <f>F22+2</f>
+        <v>2042</v>
+      </c>
       <c r="G23" s="6">
         <f t="shared" si="4"/>
         <v>2032</v>
@@ -6370,6 +6390,10 @@
       </c>
       <c r="D24" s="6" t="s">
         <v>46</v>
+      </c>
+      <c r="F24" s="6">
+        <f>F23+3</f>
+        <v>2045</v>
       </c>
       <c r="G24" s="6">
         <f t="shared" si="4"/>
@@ -6385,6 +6409,10 @@
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>
+      <c r="F25" s="6">
+        <f>F24+2</f>
+        <v>2047</v>
+      </c>
       <c r="G25" s="6">
         <f t="shared" si="4"/>
         <v>2034</v>
@@ -6399,6 +6427,10 @@
       <c r="D26" s="6" t="s">
         <v>46</v>
       </c>
+      <c r="F26" s="6">
+        <f>F25+3</f>
+        <v>2050</v>
+      </c>
       <c r="G26" s="6">
         <f t="shared" si="4"/>
         <v>2035</v>
@@ -6414,7 +6446,7 @@
         <v>46</v>
       </c>
       <c r="G27" s="6">
-        <f t="shared" ref="G27:G32" si="5">G26+2</f>
+        <f t="shared" ref="F27:G32" si="5">G26+2</f>
         <v>2037</v>
       </c>
       <c r="H27" s="6">

</xml_diff>